<commit_message>
No longer taking time lapse difference to reference twice and still experimenting with improving the phase fit
</commit_message>
<xml_diff>
--- a/TimeLapse_LaTeX/Fielddata Folder Structure.xlsx
+++ b/TimeLapse_LaTeX/Fielddata Folder Structure.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/94d3de208db0ed26/Thesis/TimeLapse_LaTeX/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/94D3DE208DB0ED26/Thesis/TimeLapse_LaTeX/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A4EE41F5-9FB2-4391-828F-765556AC49EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="148" documentId="8_{A4EE41F5-9FB2-4391-828F-765556AC49EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{34FE310A-64B0-4CA6-8FC5-596074C43A23}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BDC207CE-B99F-483C-9CB2-4F881742D5E7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="23280" windowHeight="14880" activeTab="1" xr2:uid="{BDC207CE-B99F-483C-9CB2-4F881742D5E7}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Campaigns" sheetId="1" r:id="rId1"/>
+    <sheet name="Field Notes" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="58">
   <si>
     <t>Date</t>
   </si>
@@ -174,13 +175,52 @@
   </si>
   <si>
     <t>Essentially complete for the scripted outputs</t>
+  </si>
+  <si>
+    <t>Prof #</t>
+  </si>
+  <si>
+    <t>T start</t>
+  </si>
+  <si>
+    <t>T end</t>
+  </si>
+  <si>
+    <t>Comments</t>
+  </si>
+  <si>
+    <t>prof 6 is lost</t>
+  </si>
+  <si>
+    <t>reference # 2</t>
+  </si>
+  <si>
+    <t>first after push</t>
+  </si>
+  <si>
+    <t>tracer stops at 12:47:00</t>
+  </si>
+  <si>
+    <t>chasing starts at 12:47:30</t>
+  </si>
+  <si>
+    <t>13:27:30 chasing stops</t>
+  </si>
+  <si>
+    <t>Delta T</t>
+  </si>
+  <si>
+    <t>pulling starts</t>
+  </si>
+  <si>
+    <t>Air bubbles exiting with tracer</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -201,8 +241,16 @@
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -218,6 +266,36 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2" tint="-0.749992370372631"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF67B6E"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF9F14D"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -406,7 +484,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -453,12 +531,36 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="15" fontId="1" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="21" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="21" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="21" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="21" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="20" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="21" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFF9F14D"/>
+      <color rgb="FFF67B6E"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -471,7 +573,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Kantoorthema">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1019,22 +1121,22 @@
       </c>
     </row>
     <row r="12" spans="1:6" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="10">
+      <c r="A12" s="16">
         <v>42527</v>
       </c>
-      <c r="B12" s="11">
+      <c r="B12" s="17">
         <v>2016</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="11" t="s">
+      <c r="D12" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="E12" s="11" t="s">
+      <c r="E12" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="F12" s="12" t="s">
+      <c r="F12" s="18" t="s">
         <v>34</v>
       </c>
     </row>
@@ -1116,6 +1218,642 @@
       </c>
       <c r="F16" s="15" t="s">
         <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E445BD3-A53B-4D7F-A71C-80682D0F7C32}">
+  <dimension ref="A1:E40"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" customWidth="1"/>
+    <col min="3" max="3" width="19.140625" customWidth="1"/>
+    <col min="4" max="4" width="25.5703125" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="D1" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="E1" s="19" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2" s="21">
+        <v>0.48576388888888888</v>
+      </c>
+      <c r="C2" s="21">
+        <v>0.48854166666666665</v>
+      </c>
+      <c r="D2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E2" s="20">
+        <f>C2-B2</f>
+        <v>2.7777777777777679E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" s="22">
+        <v>0.51388888888888884</v>
+      </c>
+      <c r="C3" s="22">
+        <v>0.51631944444444444</v>
+      </c>
+      <c r="D3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E3" s="20">
+        <f>C3-B3</f>
+        <v>2.4305555555556024E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" s="22">
+        <v>0.52083333333333337</v>
+      </c>
+      <c r="C4" s="22">
+        <v>0.52361111111111114</v>
+      </c>
+      <c r="E4" s="20">
+        <f t="shared" ref="E4:E40" si="0">C4-B4</f>
+        <v>2.7777777777777679E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5" s="22">
+        <v>0.52777777777777779</v>
+      </c>
+      <c r="C5" s="22">
+        <v>0.53055555555555556</v>
+      </c>
+      <c r="D5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E5" s="20">
+        <f t="shared" si="0"/>
+        <v>2.7777777777777679E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6" s="23">
+        <v>0.53472222222222221</v>
+      </c>
+      <c r="C6" s="23">
+        <v>0.53668981481481481</v>
+      </c>
+      <c r="D6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E6" s="20">
+        <f t="shared" si="0"/>
+        <v>1.9675925925926041E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>5</v>
+      </c>
+      <c r="B7" s="23">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="C7" s="23">
+        <v>0.54398148148148151</v>
+      </c>
+      <c r="E7" s="20">
+        <f t="shared" si="0"/>
+        <v>2.3148148148148806E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>6</v>
+      </c>
+      <c r="B8" s="24"/>
+      <c r="C8" s="24"/>
+      <c r="D8" t="s">
+        <v>49</v>
+      </c>
+      <c r="E8" s="20"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>7</v>
+      </c>
+      <c r="B9" s="23">
+        <v>0.54861111111111116</v>
+      </c>
+      <c r="C9" s="23">
+        <v>0.55121527777777779</v>
+      </c>
+      <c r="E9" s="20">
+        <f t="shared" si="0"/>
+        <v>2.6041666666666297E-3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>8</v>
+      </c>
+      <c r="B10" s="23">
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="C10" s="23">
+        <v>0.5581018518518519</v>
+      </c>
+      <c r="D10" t="s">
+        <v>54</v>
+      </c>
+      <c r="E10" s="20">
+        <f t="shared" si="0"/>
+        <v>2.5462962962963243E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>9</v>
+      </c>
+      <c r="B11" s="27">
+        <v>0.5625</v>
+      </c>
+      <c r="C11" s="27">
+        <v>0.56458333333333333</v>
+      </c>
+      <c r="E11" s="20">
+        <f t="shared" si="0"/>
+        <v>2.0833333333333259E-3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>10</v>
+      </c>
+      <c r="B12" s="27">
+        <v>0.56944444444444442</v>
+      </c>
+      <c r="C12" s="27">
+        <v>0.57164351851851847</v>
+      </c>
+      <c r="E12" s="20">
+        <f t="shared" si="0"/>
+        <v>2.1990740740740478E-3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>11</v>
+      </c>
+      <c r="B13" s="27">
+        <v>0.57638888888888884</v>
+      </c>
+      <c r="C13" s="27">
+        <v>0.57881944444444444</v>
+      </c>
+      <c r="E13" s="20">
+        <f t="shared" si="0"/>
+        <v>2.4305555555556024E-3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>12</v>
+      </c>
+      <c r="B14" s="27">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="C14" s="27">
+        <v>0.58599537037037042</v>
+      </c>
+      <c r="E14" s="20">
+        <f t="shared" si="0"/>
+        <v>2.6620370370370461E-3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>13</v>
+      </c>
+      <c r="B15" s="27">
+        <v>0.59027777777777779</v>
+      </c>
+      <c r="C15" s="27">
+        <v>0.59247685185185184</v>
+      </c>
+      <c r="E15" s="20">
+        <f t="shared" si="0"/>
+        <v>2.1990740740740478E-3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>14</v>
+      </c>
+      <c r="B16" s="27">
+        <v>0.59722222222222221</v>
+      </c>
+      <c r="C16" s="27">
+        <v>0.59953703703703709</v>
+      </c>
+      <c r="E16" s="20">
+        <f t="shared" si="0"/>
+        <v>2.3148148148148806E-3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>15</v>
+      </c>
+      <c r="B17" s="27">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="C17" s="27">
+        <v>0.61319444444444449</v>
+      </c>
+      <c r="E17" s="20">
+        <f t="shared" si="0"/>
+        <v>9.0277777777778567E-3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>16</v>
+      </c>
+      <c r="B18" s="27">
+        <v>0.61238425925925921</v>
+      </c>
+      <c r="C18" s="27">
+        <v>0.61498842592592595</v>
+      </c>
+      <c r="E18" s="20">
+        <f t="shared" si="0"/>
+        <v>2.6041666666667407E-3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>17</v>
+      </c>
+      <c r="B19" s="27">
+        <v>0.61875000000000002</v>
+      </c>
+      <c r="C19" s="27">
+        <v>0.62106481481481479</v>
+      </c>
+      <c r="E19" s="20">
+        <f>C19-B19</f>
+        <v>2.3148148148147696E-3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>18</v>
+      </c>
+      <c r="B20" s="27">
+        <v>0.625</v>
+      </c>
+      <c r="C20" s="27">
+        <v>0.62824074074074077</v>
+      </c>
+      <c r="E20" s="20">
+        <f t="shared" si="0"/>
+        <v>3.2407407407407662E-3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>19</v>
+      </c>
+      <c r="B21" s="27">
+        <v>0.63194444444444442</v>
+      </c>
+      <c r="C21" s="27">
+        <v>0.64606481481481481</v>
+      </c>
+      <c r="E21" s="20">
+        <f t="shared" si="0"/>
+        <v>1.4120370370370394E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>20</v>
+      </c>
+      <c r="B22" s="27">
+        <v>0.63888888888888884</v>
+      </c>
+      <c r="C22" s="27">
+        <v>0.64166666666666672</v>
+      </c>
+      <c r="E22" s="20">
+        <f t="shared" si="0"/>
+        <v>2.7777777777778789E-3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>21</v>
+      </c>
+      <c r="B23" s="25">
+        <v>0.64756944444444442</v>
+      </c>
+      <c r="C23" s="25">
+        <v>0.65011574074074074</v>
+      </c>
+      <c r="D23" t="s">
+        <v>56</v>
+      </c>
+      <c r="E23" s="20">
+        <f t="shared" si="0"/>
+        <v>2.5462962962963243E-3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>22</v>
+      </c>
+      <c r="B24" s="25">
+        <v>0.65277777777777779</v>
+      </c>
+      <c r="C24" s="25">
+        <v>0.65486111111111112</v>
+      </c>
+      <c r="E24" s="20">
+        <f t="shared" si="0"/>
+        <v>2.0833333333333259E-3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>23</v>
+      </c>
+      <c r="B25" s="25">
+        <v>0.65972222222222221</v>
+      </c>
+      <c r="C25" s="25">
+        <v>0.66192129629629626</v>
+      </c>
+      <c r="E25" s="20">
+        <f t="shared" si="0"/>
+        <v>2.1990740740740478E-3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>24</v>
+      </c>
+      <c r="B26" s="25">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="C26" s="25">
+        <v>0.66909722222222223</v>
+      </c>
+      <c r="D26" t="s">
+        <v>57</v>
+      </c>
+      <c r="E26" s="20">
+        <f t="shared" si="0"/>
+        <v>2.4305555555556024E-3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>25</v>
+      </c>
+      <c r="B27" s="25">
+        <v>0.67361111111111116</v>
+      </c>
+      <c r="C27" s="25">
+        <v>0.67754629629629626</v>
+      </c>
+      <c r="E27" s="20">
+        <f t="shared" si="0"/>
+        <v>3.9351851851850972E-3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>26</v>
+      </c>
+      <c r="B28" s="25">
+        <v>0.68194444444444446</v>
+      </c>
+      <c r="C28" s="25">
+        <v>0.68460648148148151</v>
+      </c>
+      <c r="E28" s="20">
+        <f t="shared" si="0"/>
+        <v>2.6620370370370461E-3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>27</v>
+      </c>
+      <c r="B29" s="25">
+        <v>0.6875</v>
+      </c>
+      <c r="C29" s="25">
+        <v>0.68975694444444446</v>
+      </c>
+      <c r="E29" s="20">
+        <f t="shared" si="0"/>
+        <v>2.2569444444444642E-3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>28</v>
+      </c>
+      <c r="B30" s="25">
+        <v>0.69444444444444442</v>
+      </c>
+      <c r="C30" s="25">
+        <v>0.69762731481481477</v>
+      </c>
+      <c r="E30" s="20">
+        <f t="shared" si="0"/>
+        <v>3.1828703703703498E-3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>29</v>
+      </c>
+      <c r="B31" s="25">
+        <v>0.70138888888888884</v>
+      </c>
+      <c r="C31" s="25">
+        <v>0.70416666666666672</v>
+      </c>
+      <c r="E31" s="20">
+        <f t="shared" si="0"/>
+        <v>2.7777777777778789E-3</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>30</v>
+      </c>
+      <c r="B32" s="26">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="C32" s="25">
+        <v>0.71111111111111114</v>
+      </c>
+      <c r="E32" s="20">
+        <f t="shared" si="0"/>
+        <v>2.7777777777777679E-3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>31</v>
+      </c>
+      <c r="B33" s="25">
+        <v>0.71597222222222223</v>
+      </c>
+      <c r="C33" s="25">
+        <v>0.71840277777777772</v>
+      </c>
+      <c r="E33" s="20">
+        <f t="shared" si="0"/>
+        <v>2.4305555555554914E-3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>32</v>
+      </c>
+      <c r="B34" s="25">
+        <v>0.72222222222222221</v>
+      </c>
+      <c r="C34" s="25">
+        <v>0.72465277777777781</v>
+      </c>
+      <c r="E34" s="20">
+        <f t="shared" si="0"/>
+        <v>2.4305555555556024E-3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>33</v>
+      </c>
+      <c r="B35" s="25">
+        <v>0.72916666666666663</v>
+      </c>
+      <c r="C35" s="25">
+        <v>0.7319444444444444</v>
+      </c>
+      <c r="E35" s="20">
+        <f t="shared" si="0"/>
+        <v>2.7777777777777679E-3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>34</v>
+      </c>
+      <c r="B36" s="25">
+        <v>0.73611111111111116</v>
+      </c>
+      <c r="C36" s="25">
+        <v>0.73888888888888893</v>
+      </c>
+      <c r="E36" s="20">
+        <f t="shared" si="0"/>
+        <v>2.7777777777777679E-3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>35</v>
+      </c>
+      <c r="B37" s="25">
+        <v>0.74340277777777775</v>
+      </c>
+      <c r="C37" s="25">
+        <v>0.74600694444444449</v>
+      </c>
+      <c r="E37" s="20">
+        <f t="shared" si="0"/>
+        <v>2.6041666666667407E-3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>36</v>
+      </c>
+      <c r="B38" s="25">
+        <v>0.75069444444444444</v>
+      </c>
+      <c r="C38" s="25">
+        <v>0.75335648148148149</v>
+      </c>
+      <c r="E38" s="20">
+        <f t="shared" si="0"/>
+        <v>2.6620370370370461E-3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>37</v>
+      </c>
+      <c r="B39" s="25">
+        <v>0.75694444444444442</v>
+      </c>
+      <c r="C39" s="25">
+        <v>0.75949074074074074</v>
+      </c>
+      <c r="E39" s="20">
+        <f t="shared" si="0"/>
+        <v>2.5462962962963243E-3</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>38</v>
+      </c>
+      <c r="B40" s="25">
+        <v>0.76388888888888884</v>
+      </c>
+      <c r="C40" s="25">
+        <v>0.7675925925925926</v>
+      </c>
+      <c r="E40" s="20">
+        <f t="shared" si="0"/>
+        <v>3.7037037037037646E-3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>